<commit_message>
docs: mark SN 15 complied
Delivered 29-Oct-2026, ahead of its 09-Nov start. Estimate-days still open
drop from 164 to 160.

The note records the scope caveat rather than leaving it implicit: group
membership would be the ideal source of privilege and is not forwarded, so the
serial is met from the SOC's own declaration plus observed activity and
account-name shape. If account-management events arrive later, membership
becomes a fourth and stronger signal with no redesign.

Sheet structure verified unchanged: same row count, same 26 serials, same 280
merged ranges.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UEBA Odisha Rfp Priority.xlsx
+++ b/UEBA Odisha Rfp Priority.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -220,6 +220,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1629,82 +1632,87 @@
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="53" t="inlineStr">
+      <c r="A24" s="49" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B24" s="29" t="inlineStr">
+      <c r="B24" s="48" t="inlineStr">
         <is>
           <t>UEBA</t>
         </is>
       </c>
-      <c r="C24" s="29" t="inlineStr">
+      <c r="C24" s="48" t="inlineStr">
         <is>
           <t>Aditya Umathe</t>
         </is>
       </c>
-      <c r="D24" s="53" t="inlineStr">
+      <c r="D24" s="49" t="inlineStr">
         <is>
           <t>SN 15: High privilege access anomaly detection for misuse, sharing, or takeover</t>
         </is>
       </c>
-      <c r="E24" s="29" t="inlineStr">
+      <c r="E24" s="49" t="inlineStr">
         <is>
-          <t>Can Be</t>
+          <t>Complied - DONE 29-Oct-2026</t>
         </is>
       </c>
-      <c r="F24" s="29" t="inlineStr">
+      <c r="F24" s="48" t="inlineStr">
         <is>
           <t>UEBA</t>
         </is>
       </c>
-      <c r="G24" s="53" t="n">
-        <v>4</v>
+      <c r="G24" s="49" t="n">
+        <v>0</v>
       </c>
-      <c r="H24" s="29" t="inlineStr">
+      <c r="H24" s="49" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
-      <c r="I24" s="29" t="inlineStr">
+      <c r="I24" s="48" t="inlineStr">
         <is>
           <t>Aditya, Aishwarya</t>
         </is>
       </c>
-      <c r="J24" s="30" t="n">
+      <c r="J24" s="50" t="n">
         <v>46335</v>
       </c>
-      <c r="K24" s="30" t="n">
+      <c r="K24" s="50" t="n">
         <v>46339</v>
       </c>
-      <c r="L24" s="53" t="inlineStr">
+      <c r="L24" s="49" t="inlineStr">
         <is>
-          <t>P1 - Privileged access anomaly detection.
-SN 19 is DONE (29-Oct-2026): unusual username-plus-device-plus-location combinations are detected. Presence is now recorded on every event, so 'first time this account has been seen from this country / on this host' is a real signal instead of one drawn from alerts alone. It also fixed a field path that meant the per-entity host list had never been populated at all - empty on all 155,160 profile rows.
-SN 15 remains: privilege level scored as an entity attribute so misuse, sharing or takeover of a high-privilege account is detected. The live stream does carry privilege signals to build on - 4673 failed privileged operations, plus the elevated_process and privilege_escalation rule groups. Estimate 4 d.</t>
+          <t>DONE 29-Oct-2026, ahead of the 09-Nov start.
+Privilege is now scored as an entity attribute, so an administrator's unusual behaviour surfaces sooner than a standard user's. Three named behaviours are detected: TAKEOVER (a privileged account on a host it has never used), CREDENTIAL SHARING (one human privileged account across several hosts) and MISUSE (a privileged operation outside business hours).
+The SOC declares its own privileged accounts from the console and that declaration overrides anything the system infers; where nothing is declared, the level is taken from observed privileged operations and then from the account-name shape, and every verdict records which signal produced it.
+Machine and service accounts are exempt from the sharing check because being on every host is their job. On this estate that is the difference between a usable signal and three permanent false alarms: SYSTEM is on 12 hosts, NETWORK SERVICE on 11, LOCAL SERVICE on 6. 27 entities classified on the live estate.</t>
         </is>
       </c>
-      <c r="M24" s="31" t="n"/>
-      <c r="N24" s="31" t="n"/>
-      <c r="O24" s="10" t="n"/>
-      <c r="P24" s="10" t="n"/>
-      <c r="Q24" s="10" t="n"/>
-      <c r="R24" s="10" t="n"/>
-      <c r="S24" s="10" t="n"/>
-      <c r="T24" s="10" t="n"/>
-      <c r="U24" s="10" t="n"/>
-      <c r="V24" s="10" t="n"/>
-      <c r="W24" s="10" t="n"/>
-      <c r="X24" s="10" t="n"/>
-      <c r="Y24" s="10" t="n"/>
-      <c r="Z24" s="10" t="n"/>
-      <c r="AA24" s="10" t="n"/>
-      <c r="AB24" s="10" t="n"/>
-      <c r="AC24" s="10" t="n"/>
-      <c r="AD24" s="10" t="n"/>
-      <c r="AE24" s="10" t="n"/>
-      <c r="AF24" s="10" t="n"/>
+      <c r="M24" s="57" t="inlineStr">
+        <is>
+          <t>NOTE ON SCOPE. Group membership would be the ideal source of privilege and is not forwarded by the SIEM - the same data gap that blocks SN 43 - so there is no 'Domain Admins' membership to read. The serial is met without it, from three other signals, with the SOC's own declaration taking precedence. If account-management events are forwarded later, group membership becomes a fourth and stronger signal with no redesign.</t>
+        </is>
+      </c>
+      <c r="N24" s="51" t="n"/>
+      <c r="O24" s="52" t="n"/>
+      <c r="P24" s="52" t="n"/>
+      <c r="Q24" s="52" t="n"/>
+      <c r="R24" s="52" t="n"/>
+      <c r="S24" s="52" t="n"/>
+      <c r="T24" s="52" t="n"/>
+      <c r="U24" s="52" t="n"/>
+      <c r="V24" s="52" t="n"/>
+      <c r="W24" s="52" t="n"/>
+      <c r="X24" s="52" t="n"/>
+      <c r="Y24" s="52" t="n"/>
+      <c r="Z24" s="52" t="n"/>
+      <c r="AA24" s="52" t="n"/>
+      <c r="AB24" s="52" t="n"/>
+      <c r="AC24" s="52" t="n"/>
+      <c r="AD24" s="52" t="n"/>
+      <c r="AE24" s="52" t="n"/>
+      <c r="AF24" s="52" t="n"/>
     </row>
     <row r="25" ht="42" customHeight="1">
       <c r="D25" s="29" t="inlineStr">
@@ -36032,8 +36040,8 @@
     <mergeCell ref="AB22:AB23"/>
     <mergeCell ref="Y26:Y27"/>
     <mergeCell ref="R28:R29"/>
+    <mergeCell ref="AC24:AC25"/>
     <mergeCell ref="P2:P10"/>
-    <mergeCell ref="AC24:AC25"/>
     <mergeCell ref="T35:T36"/>
     <mergeCell ref="AF42:AF44"/>
     <mergeCell ref="R15:R16"/>
@@ -36044,15 +36052,18 @@
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="F26:F27"/>
     <mergeCell ref="AA24:AA25"/>
+    <mergeCell ref="M2:M10"/>
     <mergeCell ref="X28:X29"/>
     <mergeCell ref="AF2:AF10"/>
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="R2:R10"/>
     <mergeCell ref="B15:B16"/>
+    <mergeCell ref="AF15:AF16"/>
     <mergeCell ref="AA26:AA27"/>
     <mergeCell ref="F13:F14"/>
     <mergeCell ref="AC26:AC27"/>
     <mergeCell ref="H13:H14"/>
+    <mergeCell ref="AC13:AC14"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="T13:T14"/>
     <mergeCell ref="F28:F29"/>
@@ -36092,7 +36103,6 @@
     <mergeCell ref="U2:U10"/>
     <mergeCell ref="U15:U16"/>
     <mergeCell ref="W15:W16"/>
-    <mergeCell ref="I22:I23"/>
     <mergeCell ref="N26:N27"/>
     <mergeCell ref="Y15:Y16"/>
     <mergeCell ref="E13:E14"/>
@@ -36164,7 +36174,6 @@
     <mergeCell ref="K42:K44"/>
     <mergeCell ref="M42:M44"/>
     <mergeCell ref="O42:O44"/>
-    <mergeCell ref="O28:O29"/>
     <mergeCell ref="C22:C23"/>
     <mergeCell ref="X24:X25"/>
     <mergeCell ref="AB26:AB27"/>
@@ -36209,7 +36218,6 @@
     <mergeCell ref="M26:M27"/>
     <mergeCell ref="B22:B23"/>
     <mergeCell ref="F42:F44"/>
-    <mergeCell ref="AE2:AE10"/>
     <mergeCell ref="B2:B10"/>
     <mergeCell ref="Y2:Y10"/>
     <mergeCell ref="R42:R44"/>
@@ -36238,7 +36246,9 @@
     <mergeCell ref="T2:T10"/>
     <mergeCell ref="U42:U44"/>
     <mergeCell ref="AD2:AD10"/>
+    <mergeCell ref="Z22:Z23"/>
     <mergeCell ref="AD15:AD16"/>
+    <mergeCell ref="I22:I23"/>
     <mergeCell ref="L24:L25"/>
     <mergeCell ref="C35:C36"/>
     <mergeCell ref="C26:C27"/>
@@ -36247,8 +36257,6 @@
     <mergeCell ref="X15:X16"/>
     <mergeCell ref="V15:V16"/>
     <mergeCell ref="M22:M23"/>
-    <mergeCell ref="Z22:Z23"/>
-    <mergeCell ref="AF15:AF16"/>
     <mergeCell ref="K22:K23"/>
     <mergeCell ref="O26:O27"/>
     <mergeCell ref="W26:W27"/>
@@ -36290,12 +36298,12 @@
     <mergeCell ref="L42:L44"/>
     <mergeCell ref="K24:K25"/>
     <mergeCell ref="C15:C16"/>
+    <mergeCell ref="O28:O29"/>
+    <mergeCell ref="C24:C25"/>
     <mergeCell ref="N42:N44"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="M2:M10"/>
     <mergeCell ref="Q28:Q29"/>
     <mergeCell ref="E24:E25"/>
-    <mergeCell ref="AC13:AC14"/>
+    <mergeCell ref="AE2:AE10"/>
     <mergeCell ref="X42:X44"/>
     <mergeCell ref="W24:W25"/>
     <mergeCell ref="T24:T25"/>

</xml_diff>

<commit_message>
docs: mark SN 17 and SN 40 complied
Delivered 30-Oct-2026, ahead of the 16-Nov start. Estimate-days open drop from
160 to 153.

The note records the scope limit rather than leaving it implicit: frequency of
access to a tagged asset is fully supported, but no file-path field exists
anywhere in the forwarded events, so the serial's "downloading" wording is met
by byte volume where events carry it and not at file level.

Sheet structure verified unchanged: same row count, 26 serials, 280 merges.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UEBA Odisha Rfp Priority.xlsx
+++ b/UEBA Odisha Rfp Priority.xlsx
@@ -1722,80 +1722,87 @@
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="29" t="inlineStr">
+      <c r="A26" s="48" t="inlineStr">
         <is>
           <t>17, 40</t>
         </is>
       </c>
-      <c r="B26" s="29" t="inlineStr">
+      <c r="B26" s="48" t="inlineStr">
         <is>
           <t>UEBA</t>
         </is>
       </c>
-      <c r="C26" s="29" t="inlineStr">
+      <c r="C26" s="48" t="inlineStr">
         <is>
           <t>Aditya Umathe</t>
         </is>
       </c>
-      <c r="D26" s="29" t="inlineStr">
+      <c r="D26" s="48" t="inlineStr">
         <is>
           <t>SN 17: Identifying Trusted Host and Entity Compromise instances</t>
         </is>
       </c>
-      <c r="E26" s="29" t="inlineStr">
+      <c r="E26" s="49" t="inlineStr">
         <is>
-          <t>Can Be</t>
+          <t>Complied - DONE 30-Oct-2026</t>
         </is>
       </c>
-      <c r="F26" s="29" t="inlineStr">
+      <c r="F26" s="48" t="inlineStr">
         <is>
           <t>UEBA</t>
         </is>
       </c>
-      <c r="G26" s="29" t="n">
-        <v>7</v>
+      <c r="G26" s="49" t="n">
+        <v>0</v>
       </c>
-      <c r="H26" s="29" t="inlineStr">
+      <c r="H26" s="49" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
-      <c r="I26" s="29" t="inlineStr">
+      <c r="I26" s="48" t="inlineStr">
         <is>
           <t>Aditya, Aishwarya</t>
         </is>
       </c>
-      <c r="J26" s="30" t="n">
+      <c r="J26" s="50" t="n">
         <v>46342</v>
       </c>
-      <c r="K26" s="30" t="n">
+      <c r="K26" s="50" t="n">
         <v>46346</v>
       </c>
-      <c r="L26" s="29" t="inlineStr">
+      <c r="L26" s="49" t="inlineStr">
         <is>
-          <t>P1 - Trusted hosts, entity compromise and high-value assets. By 31-Jan-2027: a trusted-host list with compromise classification, and asset-value tagging so repeated or increasing access to high-value assets is weighted up. Full estimate 7 d; all done by 31-Jan-2027.</t>
+          <t>DONE 30-Oct-2026, ahead of the 16-Nov start.
+One operator register serves both serials: an entity is tagged with a role and a value tier, and the tag changes how its events score.
+SN 17 - a host declared TRUSTED is held to a HIGHER standard, not a lower one: trust means the host is load-bearing, so anomalous behaviour on it is reported as a possible compromise.
+SN 40 - access to a tagged high-value asset is measured against what that entity normally does with that asset, so a surge is relative to its own rate rather than an absolute number. First-ever access is reported separately.</t>
         </is>
       </c>
-      <c r="M26" s="31" t="n"/>
-      <c r="N26" s="31" t="n"/>
-      <c r="O26" s="10" t="n"/>
-      <c r="P26" s="10" t="n"/>
-      <c r="Q26" s="10" t="n"/>
-      <c r="R26" s="10" t="n"/>
-      <c r="S26" s="10" t="n"/>
-      <c r="T26" s="10" t="n"/>
-      <c r="U26" s="10" t="n"/>
-      <c r="V26" s="10" t="n"/>
-      <c r="W26" s="10" t="n"/>
-      <c r="X26" s="10" t="n"/>
-      <c r="Y26" s="10" t="n"/>
-      <c r="Z26" s="10" t="n"/>
-      <c r="AA26" s="10" t="n"/>
-      <c r="AB26" s="10" t="n"/>
-      <c r="AC26" s="10" t="n"/>
-      <c r="AD26" s="10" t="n"/>
-      <c r="AE26" s="10" t="n"/>
-      <c r="AF26" s="10" t="n"/>
+      <c r="M26" s="57" t="inlineStr">
+        <is>
+          <t>SCOPE NOTE. Frequency of access is fully supported (host.name on 100% of events, destination on 97%). FILE-LEVEL download tracking is NOT: no file-path field exists anywhere in the forwarded events, so 'downloaded this document' cannot be expressed. Byte volume is used where the event carries it (about one event in six) and is a secondary signal by design. The serial is met on the frequency wording; the download wording is met only by volume, not by file.</t>
+        </is>
+      </c>
+      <c r="N26" s="51" t="n"/>
+      <c r="O26" s="52" t="n"/>
+      <c r="P26" s="52" t="n"/>
+      <c r="Q26" s="52" t="n"/>
+      <c r="R26" s="52" t="n"/>
+      <c r="S26" s="52" t="n"/>
+      <c r="T26" s="52" t="n"/>
+      <c r="U26" s="52" t="n"/>
+      <c r="V26" s="52" t="n"/>
+      <c r="W26" s="52" t="n"/>
+      <c r="X26" s="52" t="n"/>
+      <c r="Y26" s="52" t="n"/>
+      <c r="Z26" s="52" t="n"/>
+      <c r="AA26" s="52" t="n"/>
+      <c r="AB26" s="52" t="n"/>
+      <c r="AC26" s="52" t="n"/>
+      <c r="AD26" s="52" t="n"/>
+      <c r="AE26" s="52" t="n"/>
+      <c r="AF26" s="52" t="n"/>
     </row>
     <row r="27" ht="42" customHeight="1">
       <c r="D27" s="29" t="inlineStr">
@@ -36040,8 +36047,8 @@
     <mergeCell ref="AB22:AB23"/>
     <mergeCell ref="Y26:Y27"/>
     <mergeCell ref="R28:R29"/>
+    <mergeCell ref="P2:P10"/>
     <mergeCell ref="AC24:AC25"/>
-    <mergeCell ref="P2:P10"/>
     <mergeCell ref="T35:T36"/>
     <mergeCell ref="AF42:AF44"/>
     <mergeCell ref="R15:R16"/>
@@ -36058,12 +36065,10 @@
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="R2:R10"/>
     <mergeCell ref="B15:B16"/>
-    <mergeCell ref="AF15:AF16"/>
     <mergeCell ref="AA26:AA27"/>
     <mergeCell ref="F13:F14"/>
     <mergeCell ref="AC26:AC27"/>
     <mergeCell ref="H13:H14"/>
-    <mergeCell ref="AC13:AC14"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="T13:T14"/>
     <mergeCell ref="F28:F29"/>
@@ -36160,6 +36165,7 @@
     <mergeCell ref="K28:K29"/>
     <mergeCell ref="AD22:AD23"/>
     <mergeCell ref="Z15:Z16"/>
+    <mergeCell ref="E24:E25"/>
     <mergeCell ref="AB15:AB16"/>
     <mergeCell ref="S26:S27"/>
     <mergeCell ref="AF13:AF14"/>
@@ -36247,6 +36253,7 @@
     <mergeCell ref="U42:U44"/>
     <mergeCell ref="AD2:AD10"/>
     <mergeCell ref="Z22:Z23"/>
+    <mergeCell ref="AF15:AF16"/>
     <mergeCell ref="AD15:AD16"/>
     <mergeCell ref="I22:I23"/>
     <mergeCell ref="L24:L25"/>
@@ -36296,13 +36303,13 @@
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="AA13:AA14"/>
     <mergeCell ref="L42:L44"/>
+    <mergeCell ref="AC13:AC14"/>
     <mergeCell ref="K24:K25"/>
     <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C24:C25"/>
     <mergeCell ref="O28:O29"/>
-    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="Q28:Q29"/>
     <mergeCell ref="N42:N44"/>
-    <mergeCell ref="Q28:Q29"/>
-    <mergeCell ref="E24:E25"/>
     <mergeCell ref="AE2:AE10"/>
     <mergeCell ref="X42:X44"/>
     <mergeCell ref="W24:W25"/>

</xml_diff>